<commit_message>
Execute 8 workbook tests with evidence (static, secrets, config, CRUD); log run
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -5498,11 +5498,15 @@
       </c>
       <c r="N3" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O3" s="30" t="str"/>
-      <c r="P3" s="30" t="str"/>
+      <c r="P3" s="30" t="inlineStr">
+        <is>
+          <t>py_compile clean 2026-09-24 on all src/tests py (commit 793dc08); non-Qt imports OK; Qt import needs PySide6 venv</t>
+        </is>
+      </c>
       <c r="Q3" s="30" t="str"/>
       <c r="R3" s="30" t="inlineStr">
         <is>
@@ -5584,11 +5588,15 @@
       </c>
       <c r="N4" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O4" s="30" t="str"/>
-      <c r="P4" s="30" t="str"/>
+      <c r="P4" s="30" t="inlineStr">
+        <is>
+          <t>Secrets scan clean 2026-09-24: no .env/*.pem/*.key, no credentialed URLs/keys; only name-tokenizer identifiers in ingest.py</t>
+        </is>
+      </c>
       <c r="Q4" s="30" t="str"/>
       <c r="R4" s="30" t="inlineStr">
         <is>
@@ -5756,11 +5764,15 @@
       </c>
       <c r="N6" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O6" s="30" t="str"/>
-      <c r="P6" s="30" t="str"/>
+      <c r="P6" s="30" t="inlineStr">
+        <is>
+          <t>Arch audit 2026-09-24: Qt entry src/main.py, dead Tk app.py noted, resource/working-copy data flow verified</t>
+        </is>
+      </c>
       <c r="Q6" s="30" t="str"/>
       <c r="R6" s="30" t="inlineStr">
         <is>
@@ -5842,11 +5854,15 @@
       </c>
       <c r="N7" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O7" s="30" t="str"/>
-      <c r="P7" s="30" t="str"/>
+      <c r="P7" s="30" t="inlineStr">
+        <is>
+          <t>Build config verified 2026-09-24: spec entry/srcmain, datas db, version_info 3.3.0, ico, manifest all present</t>
+        </is>
+      </c>
       <c r="Q7" s="30" t="str"/>
       <c r="R7" s="30" t="inlineStr">
         <is>
@@ -6014,11 +6030,15 @@
       </c>
       <c r="N9" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O9" s="30" t="str"/>
-      <c r="P9" s="30" t="str"/>
+      <c r="P9" s="30" t="inlineStr">
+        <is>
+          <t>Fixture-DB CRUD script 2026-09-24: save_build OK (id=1)</t>
+        </is>
+      </c>
       <c r="Q9" s="30" t="str"/>
       <c r="R9" s="30" t="inlineStr">
         <is>
@@ -6100,11 +6120,15 @@
       </c>
       <c r="N10" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O10" s="30" t="str"/>
-      <c r="P10" s="30" t="str"/>
+      <c r="P10" s="30" t="inlineStr">
+        <is>
+          <t>Fixture-DB CRUD script 2026-09-24: get_build/list OK</t>
+        </is>
+      </c>
       <c r="Q10" s="30" t="str"/>
       <c r="R10" s="30" t="inlineStr">
         <is>
@@ -6186,11 +6210,15 @@
       </c>
       <c r="N11" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O11" s="30" t="str"/>
-      <c r="P11" s="30" t="str"/>
+      <c r="P11" s="30" t="inlineStr">
+        <is>
+          <t>Fixture-DB CRUD script 2026-09-24: update + duplicate OK</t>
+        </is>
+      </c>
       <c r="Q11" s="30" t="str"/>
       <c r="R11" s="30" t="inlineStr">
         <is>
@@ -6272,11 +6300,15 @@
       </c>
       <c r="N12" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O12" s="30" t="str"/>
-      <c r="P12" s="30" t="str"/>
+      <c r="P12" s="30" t="inlineStr">
+        <is>
+          <t>Fixture-DB CRUD script 2026-09-24: delete OK, 0 remaining; plus PersistenceAndImportTests 3/3 green</t>
+        </is>
+      </c>
       <c r="Q12" s="30" t="str"/>
       <c r="R12" s="30" t="inlineStr">
         <is>
@@ -19542,20 +19574,68 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="29" t="str"/>
-      <c r="B4" s="30" t="str"/>
-      <c r="C4" s="30" t="str"/>
-      <c r="D4" s="30" t="str"/>
-      <c r="E4" s="30" t="str"/>
-      <c r="F4" s="30" t="str"/>
-      <c r="G4" s="30" t="str"/>
-      <c r="H4" s="30" t="str"/>
-      <c r="I4" s="30" t="str"/>
-      <c r="J4" s="30" t="str"/>
-      <c r="K4" s="30" t="str"/>
-      <c r="L4" s="30" t="str"/>
-      <c r="M4" s="30" t="str"/>
-      <c r="N4" s="31" t="str"/>
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260924-EXEC</t>
+        </is>
+      </c>
+      <c r="B4" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t>main 793dc08</t>
+        </is>
+      </c>
+      <c r="D4" s="30" t="inlineStr">
+        <is>
+          <t>Windows x64 / seed+fixture DB</t>
+        </is>
+      </c>
+      <c r="E4" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11 / Python 3.13</t>
+        </is>
+      </c>
+      <c r="F4" s="30" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G4" s="30" t="inlineStr">
+        <is>
+          <t>manager</t>
+        </is>
+      </c>
+      <c r="H4" s="30" t="inlineStr">
+        <is>
+          <t>T001 py_compile, T002 secrets scan, T004/T005 config audit, T007-T010 fixture CRUD</t>
+        </is>
+      </c>
+      <c r="I4" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="J4" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="K4" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="30" t="inlineStr">
+        <is>
+          <t>~5min</t>
+        </is>
+      </c>
+      <c r="N4" s="31" t="inlineStr">
+        <is>
+          <t>T003 vuln DB (no pip-audit) and T006 clean EXE build left NOT STARTED</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="29" t="str"/>

</xml_diff>

<commit_message>
Qt offscreen smoke test, T003 pip-audit PASS, 9 workbook tests green
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -5678,11 +5678,15 @@
       </c>
       <c r="N5" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O5" s="30" t="str"/>
-      <c r="P5" s="30" t="str"/>
+      <c r="P5" s="30" t="inlineStr">
+        <is>
+          <t>pip-audit 2.10.1 on requirements.txt 2026-09-24: No known vulnerabilities found (PySide6==6.9.1)</t>
+        </is>
+      </c>
       <c r="Q5" s="30" t="str"/>
       <c r="R5" s="30" t="inlineStr">
         <is>
@@ -19638,20 +19642,68 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="str"/>
-      <c r="B5" s="30" t="str"/>
-      <c r="C5" s="30" t="str"/>
-      <c r="D5" s="30" t="str"/>
-      <c r="E5" s="30" t="str"/>
-      <c r="F5" s="30" t="str"/>
-      <c r="G5" s="30" t="str"/>
-      <c r="H5" s="30" t="str"/>
-      <c r="I5" s="30" t="str"/>
-      <c r="J5" s="30" t="str"/>
-      <c r="K5" s="30" t="str"/>
-      <c r="L5" s="30" t="str"/>
-      <c r="M5" s="30" t="str"/>
-      <c r="N5" s="31" t="str"/>
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260924-AUDIT2</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>main 61611b8</t>
+        </is>
+      </c>
+      <c r="D5" s="30" t="inlineStr">
+        <is>
+          <t>Windows x64 / .venv PySide6 6.9.1 offscreen</t>
+        </is>
+      </c>
+      <c r="E5" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11 / Python 3.13</t>
+        </is>
+      </c>
+      <c r="F5" s="30" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G5" s="30" t="inlineStr">
+        <is>
+          <t>manager</t>
+        </is>
+      </c>
+      <c r="H5" s="30" t="inlineStr">
+        <is>
+          <t>T003 pip-audit clean; Qt offscreen smoke 2/2 (8 tabs, title); full suite 13 pass / 6 blocked on seed DB</t>
+        </is>
+      </c>
+      <c r="I5" s="30" t="n">
+        <v>19</v>
+      </c>
+      <c r="J5" s="30" t="n">
+        <v>13</v>
+      </c>
+      <c r="K5" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="30" t="n">
+        <v>6</v>
+      </c>
+      <c r="M5" s="30" t="inlineStr">
+        <is>
+          <t>~3min</t>
+        </is>
+      </c>
+      <c r="N5" s="31" t="inlineStr">
+        <is>
+          <t>6 blocked unchanged: production DB only in private release</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="29" t="str"/>

</xml_diff>

<commit_message>
Agent-H S3 extension and sweep hardening; T006 build PASS with evidence
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -5948,11 +5948,15 @@
       </c>
       <c r="N8" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O8" s="30" t="str"/>
-      <c r="P8" s="30" t="str"/>
+      <c r="P8" s="30" t="inlineStr">
+        <is>
+          <t>PyInstaller 6.22.3 build 2026-09-24 exit 0 in 33s: dist/Propeller_Calculator_Professional_UA_v3_3.exe 47.8MB, icon/manifest/version embedded, no release-relevant warnings. Caveat: bundles seed DB (0 models); production-DB build awaits release zip.</t>
+        </is>
+      </c>
       <c r="Q8" s="30" t="str"/>
       <c r="R8" s="30" t="inlineStr">
         <is>
@@ -19706,20 +19710,68 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="str"/>
-      <c r="B6" s="30" t="str"/>
-      <c r="C6" s="30" t="str"/>
-      <c r="D6" s="30" t="str"/>
-      <c r="E6" s="30" t="str"/>
-      <c r="F6" s="30" t="str"/>
-      <c r="G6" s="30" t="str"/>
-      <c r="H6" s="30" t="str"/>
-      <c r="I6" s="30" t="str"/>
-      <c r="J6" s="30" t="str"/>
-      <c r="K6" s="30" t="str"/>
-      <c r="L6" s="30" t="str"/>
-      <c r="M6" s="30" t="str"/>
-      <c r="N6" s="31" t="str"/>
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260924-BUILD</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>main 69fe4f5</t>
+        </is>
+      </c>
+      <c r="D6" s="30" t="inlineStr">
+        <is>
+          <t>Windows x64 / .venv PyInstaller 6.22.3</t>
+        </is>
+      </c>
+      <c r="E6" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11 / Python 3.13</t>
+        </is>
+      </c>
+      <c r="F6" s="30" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G6" s="30" t="inlineStr">
+        <is>
+          <t>agent-F</t>
+        </is>
+      </c>
+      <c r="H6" s="30" t="inlineStr">
+        <is>
+          <t>T006 clean EXE build exit 0, 47.8MB; warn-file benign only</t>
+        </is>
+      </c>
+      <c r="I6" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="30" t="inlineStr">
+        <is>
+          <t>~1min</t>
+        </is>
+      </c>
+      <c r="N6" s="31" t="inlineStr">
+        <is>
+          <t>Agent report ses_F; tree left clean, no commit by agent</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="29" t="str"/>

</xml_diff>

<commit_message>
Production DB restored, full suite 19/19 green, run logged
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -19774,20 +19774,68 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="29" t="str"/>
-      <c r="B7" s="30" t="str"/>
-      <c r="C7" s="30" t="str"/>
-      <c r="D7" s="30" t="str"/>
-      <c r="E7" s="30" t="str"/>
-      <c r="F7" s="30" t="str"/>
-      <c r="G7" s="30" t="str"/>
-      <c r="H7" s="30" t="str"/>
-      <c r="I7" s="30" t="str"/>
-      <c r="J7" s="30" t="str"/>
-      <c r="K7" s="30" t="str"/>
-      <c r="L7" s="30" t="str"/>
-      <c r="M7" s="30" t="str"/>
-      <c r="N7" s="31" t="str"/>
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260924-FULLSUITE</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>main 5609ce8 + restored prod DB</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>Windows x64 / prod DB 1053 models 335434 points</t>
+        </is>
+      </c>
+      <c r="E7" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11 / Python 3.13 / .venv PySide6 6.9.1</t>
+        </is>
+      </c>
+      <c r="F7" s="30" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G7" s="30" t="inlineStr">
+        <is>
+          <t>manager</t>
+        </is>
+      </c>
+      <c r="H7" s="30" t="inlineStr">
+        <is>
+          <t>unittest discover: 19/19 OK incl 6 previously DB-blocked (static/dynamic/water/battery/point-mode/counts)</t>
+        </is>
+      </c>
+      <c r="I7" s="30" t="n">
+        <v>19</v>
+      </c>
+      <c r="J7" s="30" t="n">
+        <v>19</v>
+      </c>
+      <c r="K7" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="30" t="inlineStr">
+        <is>
+          <t>~2s</t>
+        </is>
+      </c>
+      <c r="N7" s="31" t="inlineStr">
+        <is>
+          <t>DB zip 92.6MB from private release; seed DB preserved as work/build/propellers.seed.db</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="29" t="str"/>

</xml_diff>

<commit_message>
Agent wave results: UI 14/14, calc exact, 15 workbook PASS with evidence
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -6656,11 +6656,15 @@
       </c>
       <c r="N16" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O16" s="30" t="str"/>
-      <c r="P16" s="30" t="str"/>
+      <c r="P16" s="30" t="inlineStr">
+        <is>
+          <t>Boundary sweep 2026-09-24 (probe2, prod copy): 0/neg/max/decimal/huge/NaN/Inf all guarded, warnings match domain rules; guard suite green</t>
+        </is>
+      </c>
       <c r="Q16" s="30" t="str"/>
       <c r="R16" s="30" t="inlineStr">
         <is>
@@ -6828,11 +6832,15 @@
       </c>
       <c r="N18" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O18" s="30" t="str"/>
-      <c r="P18" s="30" t="str"/>
+      <c r="P18" s="30" t="inlineStr">
+        <is>
+          <t>units round-trip 11/11 exact to 1e-10 + UI SI-Imperial invariance 18.25613624 N identical (UI test si_imperial_si PASS)</t>
+        </is>
+      </c>
       <c r="Q18" s="30" t="str"/>
       <c r="R18" s="30" t="inlineStr">
         <is>
@@ -6914,11 +6922,15 @@
       </c>
       <c r="N19" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O19" s="30" t="str"/>
-      <c r="P19" s="30" t="str"/>
+      <c r="P19" s="30" t="inlineStr">
+        <is>
+          <t>Suite test_merge_is_idempotent_then_updates_and_adds OK: idempotent, update, add paths + 3 backups/history</t>
+        </is>
+      </c>
       <c r="Q19" s="30" t="str"/>
       <c r="R19" s="30" t="inlineStr">
         <is>
@@ -7000,11 +7012,15 @@
       </c>
       <c r="N20" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O20" s="30" t="str"/>
-      <c r="P20" s="30" t="str"/>
+      <c r="P20" s="30" t="inlineStr">
+        <is>
+          <t>Corrupt-import probe 2026-09-24: empty/trunc zip BadZipFile, wrong ext rejected, bad CSV flagged; counts 1053/335434 unchanged, quick_check ok</t>
+        </is>
+      </c>
       <c r="Q20" s="30" t="str"/>
       <c r="R20" s="30" t="inlineStr">
         <is>
@@ -7086,11 +7102,15 @@
       </c>
       <c r="N21" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O21" s="30" t="str"/>
-      <c r="P21" s="30" t="str"/>
+      <c r="P21" s="30" t="inlineStr">
+        <is>
+          <t>32MB unrecognized zip rejected gracefully (ImportErrorWithReport) in 0.9s, no crash, models still 1053</t>
+        </is>
+      </c>
       <c r="Q21" s="30" t="str"/>
       <c r="R21" s="30" t="inlineStr">
         <is>
@@ -7172,11 +7192,15 @@
       </c>
       <c r="N22" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O22" s="30" t="n"/>
-      <c r="P22" s="30" t="n"/>
+      <c r="P22" s="30" t="inlineStr">
+        <is>
+          <t>Unicode-path probe: space/Cyrillic/emoji/120-char dirs, import+export OK, 1053 models each</t>
+        </is>
+      </c>
       <c r="Q22" s="30" t="n"/>
       <c r="R22" s="30" t="inlineStr">
         <is>
@@ -7258,11 +7282,15 @@
       </c>
       <c r="N23" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O23" s="30" t="str"/>
-      <c r="P23" s="30" t="str"/>
+      <c r="P23" s="30" t="inlineStr">
+        <is>
+          <t>3 DB exports byte-identical (sha 66ded93d...), 1053 models/335434 points each = source values preserved</t>
+        </is>
+      </c>
       <c r="Q23" s="30" t="str"/>
       <c r="R23" s="30" t="inlineStr">
         <is>
@@ -7344,11 +7372,15 @@
       </c>
       <c r="N24" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O24" s="30" t="str"/>
-      <c r="P24" s="30" t="str"/>
+      <c r="P24" s="30" t="inlineStr">
+        <is>
+          <t>Repeat-export 3/3 deterministic identical artifacts, no state leak (10x loop proposed, 3x evidenced)</t>
+        </is>
+      </c>
       <c r="Q24" s="30" t="str"/>
       <c r="R24" s="30" t="inlineStr">
         <is>
@@ -7688,11 +7720,15 @@
       </c>
       <c r="N28" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O28" s="30" t="n"/>
-      <c r="P28" s="30" t="n"/>
+      <c r="P28" s="30" t="inlineStr">
+        <is>
+          <t>Zero network calls in src (grep audit) + offscreen cold start 0.61s on prod DB, 8 tabs accessible; offline by design</t>
+        </is>
+      </c>
       <c r="Q28" s="30" t="n"/>
       <c r="R28" s="30" t="inlineStr">
         <is>
@@ -7774,11 +7810,15 @@
       </c>
       <c r="N29" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O29" s="30" t="str"/>
-      <c r="P29" s="30" t="str"/>
+      <c r="P29" s="30" t="inlineStr">
+        <is>
+          <t>Suite persistence tests OK: save-close-reopen round-trip + accessory inventory on local sqlite (offline path)</t>
+        </is>
+      </c>
       <c r="Q29" s="30" t="str"/>
       <c r="R29" s="30" t="inlineStr">
         <is>
@@ -8204,11 +8244,15 @@
       </c>
       <c r="N34" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O34" s="30" t="n"/>
-      <c r="P34" s="30" t="n"/>
+      <c r="P34" s="30" t="inlineStr">
+        <is>
+          <t>6 injection payloads via parameterized search: 0 rows, stored as data, models intact; no execution</t>
+        </is>
+      </c>
       <c r="Q34" s="30" t="n"/>
       <c r="R34" s="30" t="inlineStr">
         <is>
@@ -9494,11 +9538,15 @@
       </c>
       <c r="N49" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O49" s="30" t="n"/>
-      <c r="P49" s="30" t="n"/>
+      <c r="P49" s="30" t="inlineStr">
+        <is>
+          <t>Suite: 8X9 point-mode exact (dCt=dCp=dP=0), static/dynamic air, raw-vs-interp separation all OK on prod DB</t>
+        </is>
+      </c>
       <c r="Q49" s="30" t="n"/>
       <c r="R49" s="30" t="inlineStr">
         <is>
@@ -9580,11 +9628,15 @@
       </c>
       <c r="N50" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O50" s="30" t="str"/>
-      <c r="P50" s="30" t="str"/>
+      <c r="P50" s="30" t="inlineStr">
+        <is>
+          <t>Warning probes on prod copy: ESC exceeded, C-rating exceeded, 6S mismatch 14.80 vs 22.20 V, cavitation warning all fire; sweep blocks overloads</t>
+        </is>
+      </c>
       <c r="Q50" s="30" t="str"/>
       <c r="R50" s="30" t="inlineStr">
         <is>
@@ -9752,11 +9804,15 @@
       </c>
       <c r="N52" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O52" s="30" t="n"/>
-      <c r="P52" s="30" t="n"/>
+      <c r="P52" s="30" t="inlineStr">
+        <is>
+          <t>Frozen suite 19/19 OK 2026-09-24 (RUN-20260924-FULLSUITE): 17 headless + 2 Qt offscreen</t>
+        </is>
+      </c>
       <c r="Q52" s="30" t="n"/>
       <c r="R52" s="30" t="inlineStr">
         <is>
@@ -10698,11 +10754,15 @@
       </c>
       <c r="N63" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O63" s="30" t="str"/>
-      <c r="P63" s="30" t="str"/>
+      <c r="P63" s="30" t="inlineStr">
+        <is>
+          <t>Long/emoji/multiline strings via input setters: saved/searched intact, no crash; validation warnings fire (clipboard-event path residual)</t>
+        </is>
+      </c>
       <c r="Q63" s="30" t="str"/>
       <c r="R63" s="30" t="inlineStr">
         <is>
@@ -19838,20 +19898,68 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="str"/>
-      <c r="B8" s="30" t="str"/>
-      <c r="C8" s="30" t="str"/>
-      <c r="D8" s="30" t="str"/>
-      <c r="E8" s="30" t="str"/>
-      <c r="F8" s="30" t="str"/>
-      <c r="G8" s="30" t="str"/>
-      <c r="H8" s="30" t="str"/>
-      <c r="I8" s="30" t="str"/>
-      <c r="J8" s="30" t="str"/>
-      <c r="K8" s="30" t="str"/>
-      <c r="L8" s="30" t="str"/>
-      <c r="M8" s="30" t="str"/>
-      <c r="N8" s="31" t="str"/>
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260924-WAVE</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>main 2981013 + prod DB</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>Windows x64 / prod DB copy + temp DBs</t>
+        </is>
+      </c>
+      <c r="E8" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11 / Python 3.13 / .venv</t>
+        </is>
+      </c>
+      <c r="F8" s="30" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G8" s="30" t="inlineStr">
+        <is>
+          <t>agents E/C2/D2</t>
+        </is>
+      </c>
+      <c r="H8" s="30" t="inlineStr">
+        <is>
+          <t>UI 14/14, calc numbers confirmed exact, 15 workbook PASS; T012/T013/T015/T033/T034/T037/T038/T043 need more evidence</t>
+        </is>
+      </c>
+      <c r="I8" s="30" t="n">
+        <v>15</v>
+      </c>
+      <c r="J8" s="30" t="n">
+        <v>15</v>
+      </c>
+      <c r="K8" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="30" t="inlineStr">
+        <is>
+          <t>~30min</t>
+        </is>
+      </c>
+      <c r="N8" s="31" t="inlineStr">
+        <is>
+          <t>Agent reports ses_E/C2/D2; deferred rows documented</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="29" t="str"/>

</xml_diff>

<commit_message>
10 network/browser tests N/A per user scope decision
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -7900,15 +7900,19 @@
       </c>
       <c r="N30" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O30" s="30" t="n"/>
-      <c r="P30" s="30" t="n"/>
+      <c r="P30" s="30" t="inlineStr">
+        <is>
+          <t>N/A per user decision 2026-09-24: offline Qt desktop has no network/API/session/browser layer (zero network calls in src; no server, auth, sync, or web build). No test target.</t>
+        </is>
+      </c>
       <c r="Q30" s="30" t="n"/>
       <c r="R30" s="30" t="inlineStr">
         <is>
-          <t>NOT TESTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S30" s="30" t="n"/>
@@ -7986,15 +7990,19 @@
       </c>
       <c r="N31" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O31" s="30" t="n"/>
-      <c r="P31" s="30" t="n"/>
+      <c r="P31" s="30" t="inlineStr">
+        <is>
+          <t>N/A per user decision 2026-09-24: offline Qt desktop has no network/API/session/browser layer (zero network calls in src; no server, auth, sync, or web build). No test target.</t>
+        </is>
+      </c>
       <c r="Q31" s="30" t="n"/>
       <c r="R31" s="30" t="inlineStr">
         <is>
-          <t>NOT TESTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S31" s="30" t="n"/>
@@ -8072,15 +8080,19 @@
       </c>
       <c r="N32" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O32" s="30" t="n"/>
-      <c r="P32" s="30" t="n"/>
+      <c r="P32" s="30" t="inlineStr">
+        <is>
+          <t>N/A per user decision 2026-09-24: offline Qt desktop has no network/API/session/browser layer (zero network calls in src; no server, auth, sync, or web build). No test target.</t>
+        </is>
+      </c>
       <c r="Q32" s="30" t="n"/>
       <c r="R32" s="30" t="inlineStr">
         <is>
-          <t>NOT TESTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S32" s="30" t="n"/>
@@ -8158,15 +8170,19 @@
       </c>
       <c r="N33" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O33" s="30" t="n"/>
-      <c r="P33" s="30" t="n"/>
+      <c r="P33" s="30" t="inlineStr">
+        <is>
+          <t>N/A per user decision 2026-09-24: offline Qt desktop has no network/API/session/browser layer (zero network calls in src; no server, auth, sync, or web build). No test target.</t>
+        </is>
+      </c>
       <c r="Q33" s="30" t="n"/>
       <c r="R33" s="30" t="inlineStr">
         <is>
-          <t>NOT TESTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S33" s="30" t="n"/>
@@ -8506,15 +8522,19 @@
       </c>
       <c r="N37" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O37" s="30" t="n"/>
-      <c r="P37" s="30" t="n"/>
+      <c r="P37" s="30" t="inlineStr">
+        <is>
+          <t>N/A per user decision 2026-09-24: offline Qt desktop has no network/API/session/browser layer (zero network calls in src; no server, auth, sync, or web build). No test target.</t>
+        </is>
+      </c>
       <c r="Q37" s="30" t="n"/>
       <c r="R37" s="30" t="inlineStr">
         <is>
-          <t>NOT TESTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S37" s="30" t="n"/>
@@ -8592,15 +8612,19 @@
       </c>
       <c r="N38" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O38" s="30" t="n"/>
-      <c r="P38" s="30" t="n"/>
+      <c r="P38" s="30" t="inlineStr">
+        <is>
+          <t>N/A per user decision 2026-09-24: offline Qt desktop has no network/API/session/browser layer (zero network calls in src; no server, auth, sync, or web build). No test target.</t>
+        </is>
+      </c>
       <c r="Q38" s="30" t="n"/>
       <c r="R38" s="30" t="inlineStr">
         <is>
-          <t>NOT TESTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S38" s="30" t="n"/>
@@ -9894,15 +9918,19 @@
       </c>
       <c r="N53" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O53" s="30" t="str"/>
-      <c r="P53" s="30" t="str"/>
+      <c r="P53" s="30" t="inlineStr">
+        <is>
+          <t>N/A per user decision 2026-09-24: offline Qt desktop has no network/API/session/browser layer (zero network calls in src; no server, auth, sync, or web build). No test target.</t>
+        </is>
+      </c>
       <c r="Q53" s="30" t="str"/>
       <c r="R53" s="30" t="inlineStr">
         <is>
-          <t>NOT TESTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S53" s="30" t="str"/>
@@ -9980,15 +10008,19 @@
       </c>
       <c r="N54" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O54" s="30" t="str"/>
-      <c r="P54" s="30" t="str"/>
+      <c r="P54" s="30" t="inlineStr">
+        <is>
+          <t>N/A per user decision 2026-09-24: offline Qt desktop has no network/API/session/browser layer (zero network calls in src; no server, auth, sync, or web build). No test target.</t>
+        </is>
+      </c>
       <c r="Q54" s="30" t="str"/>
       <c r="R54" s="30" t="inlineStr">
         <is>
-          <t>NOT TESTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S54" s="30" t="str"/>
@@ -10066,15 +10098,19 @@
       </c>
       <c r="N55" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O55" s="30" t="str"/>
-      <c r="P55" s="30" t="str"/>
+      <c r="P55" s="30" t="inlineStr">
+        <is>
+          <t>N/A per user decision 2026-09-24: offline Qt desktop has no network/API/session/browser layer (zero network calls in src; no server, auth, sync, or web build). No test target.</t>
+        </is>
+      </c>
       <c r="Q55" s="30" t="str"/>
       <c r="R55" s="30" t="inlineStr">
         <is>
-          <t>NOT TESTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S55" s="30" t="str"/>
@@ -11532,15 +11568,19 @@
       </c>
       <c r="N72" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O72" s="30" t="str"/>
-      <c r="P72" s="30" t="str"/>
+      <c r="P72" s="30" t="inlineStr">
+        <is>
+          <t>N/A per user decision 2026-09-24: offline Qt desktop has no network/API/session/browser layer (zero network calls in src; no server, auth, sync, or web build). No test target.</t>
+        </is>
+      </c>
       <c r="Q72" s="30" t="str"/>
       <c r="R72" s="30" t="inlineStr">
         <is>
-          <t>NOT TESTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S72" s="30" t="str"/>

</xml_diff>

<commit_message>
Probe results: P007/T015/T039 PASS, T023 N/A, widget-leak recorded
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -6746,11 +6746,15 @@
       </c>
       <c r="N17" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O17" s="30" t="str"/>
-      <c r="P17" s="30" t="str"/>
+      <c r="P17" s="30" t="inlineStr">
+        <is>
+          <t>Offscreen probe 2026-09-24: UKR-&gt;ENG via header slot, fresh read app_settings= en, 2nd instance starts ENG, 8/8 tabs English, zero Cyrillic headers</t>
+        </is>
+      </c>
       <c r="Q17" s="30" t="str"/>
       <c r="R17" s="30" t="inlineStr">
         <is>
@@ -7462,15 +7466,19 @@
       </c>
       <c r="N25" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O25" s="30" t="str"/>
-      <c r="P25" s="30" t="str"/>
+      <c r="P25" s="30" t="inlineStr">
+        <is>
+          <t>No pre-v3 schema ever existed (single commit, SCHEMA_VERSION=3 from start, zero migration/ALTER code in src); migration condition cannot occur. Agent B2 report.</t>
+        </is>
+      </c>
       <c r="Q25" s="30" t="str"/>
       <c r="R25" s="30" t="inlineStr">
         <is>
-          <t>NOT TESTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S25" s="30" t="str"/>
@@ -8874,11 +8882,15 @@
       </c>
       <c r="N41" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O41" s="30" t="n"/>
-      <c r="P41" s="30" t="n"/>
+      <c r="P41" s="30" t="inlineStr">
+        <is>
+          <t>Synthetic 2x DB (2106 models/670868 pts, FK ok): summary 48.7ms, search 27.8ms, points 2.6ms, calc 10.1ms, sweep 9.8ms; no crash, absolute times interactive</t>
+        </is>
+      </c>
       <c r="Q41" s="30" t="n"/>
       <c r="R41" s="30" t="inlineStr">
         <is>
@@ -10446,11 +10458,15 @@
       </c>
       <c r="N59" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O59" s="30" t="str"/>
-      <c r="P59" s="30" t="str"/>
+      <c r="P59" s="30" t="inlineStr">
+        <is>
+          <t>Offscreen resize 1920-640px: stacking triggers &lt;900, compact header, 8 tabs reachable, inputs visible, grab ok; min clamp 640x360 by design</t>
+        </is>
+      </c>
       <c r="Q59" s="30" t="str"/>
       <c r="R59" s="30" t="inlineStr">
         <is>
@@ -20002,20 +20018,68 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="str"/>
-      <c r="B9" s="30" t="str"/>
-      <c r="C9" s="30" t="str"/>
-      <c r="D9" s="30" t="str"/>
-      <c r="E9" s="30" t="str"/>
-      <c r="F9" s="30" t="str"/>
-      <c r="G9" s="30" t="str"/>
-      <c r="H9" s="30" t="str"/>
-      <c r="I9" s="30" t="str"/>
-      <c r="J9" s="30" t="str"/>
-      <c r="K9" s="30" t="str"/>
-      <c r="L9" s="30" t="str"/>
-      <c r="M9" s="30" t="str"/>
-      <c r="N9" s="31" t="str"/>
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260924-PROBES</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>main b34ba28 + prod DB</t>
+        </is>
+      </c>
+      <c r="D9" s="30" t="inlineStr">
+        <is>
+          <t>Windows x64 / temp DB copies</t>
+        </is>
+      </c>
+      <c r="E9" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11 / .venv offscreen</t>
+        </is>
+      </c>
+      <c r="F9" s="30" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G9" s="30" t="inlineStr">
+        <is>
+          <t>agents E2/B2</t>
+        </is>
+      </c>
+      <c r="H9" s="30" t="inlineStr">
+        <is>
+          <t>P007 resize PASS, T015 persist PASS, T023 no-upgrade-path N/A, T039 2x timings; incidental: hidden widget-tree leak on lang switch (recorded, unfixed)</t>
+        </is>
+      </c>
+      <c r="I9" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K9" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="30" t="inlineStr">
+        <is>
+          <t>~20min</t>
+        </is>
+      </c>
+      <c r="N9" s="31" t="inlineStr">
+        <is>
+          <t>Agent reports ses_E2/B2</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="29" t="str"/>

</xml_diff>

<commit_message>
Fix hidden widget-tree leak on UI rebuild; leak regression test; suite 20/20
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -20082,20 +20082,68 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="str"/>
-      <c r="B10" s="30" t="str"/>
-      <c r="C10" s="30" t="str"/>
-      <c r="D10" s="30" t="str"/>
-      <c r="E10" s="30" t="str"/>
-      <c r="F10" s="30" t="str"/>
-      <c r="G10" s="30" t="str"/>
-      <c r="H10" s="30" t="str"/>
-      <c r="I10" s="30" t="str"/>
-      <c r="J10" s="30" t="str"/>
-      <c r="K10" s="30" t="str"/>
-      <c r="L10" s="30" t="str"/>
-      <c r="M10" s="30" t="str"/>
-      <c r="N10" s="31" t="str"/>
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260924-LEAKFIX</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>main f6d985b + agent H3 fix</t>
+        </is>
+      </c>
+      <c r="D10" s="30" t="inlineStr">
+        <is>
+          <t>Windows x64 / seed DB temp copy</t>
+        </is>
+      </c>
+      <c r="E10" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11 / .venv offscreen</t>
+        </is>
+      </c>
+      <c r="F10" s="30" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G10" s="30" t="inlineStr">
+        <is>
+          <t>agent H3</t>
+        </is>
+      </c>
+      <c r="H10" s="30" t="inlineStr">
+        <is>
+          <t>Widget-tree leak fixed (takeCentralWidget+deleteLater, statusbar reuse); leak test 6-6-6; full suite 20/20 OK</t>
+        </is>
+      </c>
+      <c r="I10" s="30" t="n">
+        <v>20</v>
+      </c>
+      <c r="J10" s="30" t="n">
+        <v>20</v>
+      </c>
+      <c r="K10" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="30" t="inlineStr">
+        <is>
+          <t>~10min</t>
+        </is>
+      </c>
+      <c r="N10" s="31" t="inlineStr">
+        <is>
+          <t>Agent report ses_H3; manager verified</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="29" t="str"/>

</xml_diff>

<commit_message>
Robustness probes: T011/T024/T025/P015 PASS with evidence
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -6398,11 +6398,15 @@
       </c>
       <c r="N13" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O13" s="30" t="str"/>
-      <c r="P13" s="30" t="str"/>
+      <c r="P13" s="30" t="inlineStr">
+        <is>
+          <t>Double-save probe 2026-09-24: 2 rapid clicks = +2 builds exactly (1:1, no signal duplicates), 9/9 components, quick_check ok, 0 errors</t>
+        </is>
+      </c>
       <c r="Q13" s="30" t="str"/>
       <c r="R13" s="30" t="inlineStr">
         <is>
@@ -7556,11 +7560,15 @@
       </c>
       <c r="N26" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O26" s="30" t="str"/>
-      <c r="P26" s="30" t="str"/>
+      <c r="P26" s="30" t="inlineStr">
+        <is>
+          <t>Kill-mid-save probe: child terminated mid-TX, full rollback (0 builds/0 orphans), quick_check ok, app reopens 8 tabs</t>
+        </is>
+      </c>
       <c r="Q26" s="30" t="str"/>
       <c r="R26" s="30" t="inlineStr">
         <is>
@@ -7642,11 +7650,15 @@
       </c>
       <c r="N27" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O27" s="30" t="str"/>
-      <c r="P27" s="30" t="str"/>
+      <c r="P27" s="30" t="inlineStr">
+        <is>
+          <t>Kill-mid-import probe: only committed saves survive (3510), 0 orphans/partial, quick_check ok; single-commit atomicity (repo 248-297) + WAL</t>
+        </is>
+      </c>
       <c r="Q27" s="30" t="str"/>
       <c r="R27" s="30" t="inlineStr">
         <is>
@@ -9327,7 +9339,11 @@
           <t>NOT TESTED</t>
         </is>
       </c>
-      <c r="S46" s="30" t="n"/>
+      <c r="S46" s="30" t="inlineStr">
+        <is>
+          <t>Partial 2026-09-24: 5 rapid clicks serialize (7.65s), single result, no dup/hang; loading-indicator leg still unverified</t>
+        </is>
+      </c>
       <c r="T46" s="31" t="inlineStr">
         <is>
           <t>Before MVP</t>
@@ -11154,11 +11170,15 @@
       </c>
       <c r="N67" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O67" s="30" t="str"/>
-      <c r="P67" s="30" t="str"/>
+      <c r="P67" s="30" t="inlineStr">
+        <is>
+          <t>Whole session runs at Medium integrity (standard user, whoami 2026-09-24): suite, UI, build, DB all green with zero elevation prompts</t>
+        </is>
+      </c>
       <c r="Q67" s="30" t="str"/>
       <c r="R67" s="30" t="inlineStr">
         <is>
@@ -20146,20 +20166,68 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="str"/>
-      <c r="B11" s="30" t="str"/>
-      <c r="C11" s="30" t="str"/>
-      <c r="D11" s="30" t="str"/>
-      <c r="E11" s="30" t="str"/>
-      <c r="F11" s="30" t="str"/>
-      <c r="G11" s="30" t="str"/>
-      <c r="H11" s="30" t="str"/>
-      <c r="I11" s="30" t="str"/>
-      <c r="J11" s="30" t="str"/>
-      <c r="K11" s="30" t="str"/>
-      <c r="L11" s="30" t="str"/>
-      <c r="M11" s="30" t="str"/>
-      <c r="N11" s="31" t="str"/>
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260924-ROBUST</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>main fb7b3e9 + prod DB</t>
+        </is>
+      </c>
+      <c r="D11" s="30" t="inlineStr">
+        <is>
+          <t>Windows x64 / temp DB copies</t>
+        </is>
+      </c>
+      <c r="E11" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11 / .venv offscreen</t>
+        </is>
+      </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G11" s="30" t="inlineStr">
+        <is>
+          <t>agent G + manager(P015)</t>
+        </is>
+      </c>
+      <c r="H11" s="30" t="inlineStr">
+        <is>
+          <t>T011/T024/T025/P015 PASS; T044 partial (loading leg open)</t>
+        </is>
+      </c>
+      <c r="I11" s="30" t="n">
+        <v>5</v>
+      </c>
+      <c r="J11" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="K11" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="30" t="inlineStr">
+        <is>
+          <t>~25min</t>
+        </is>
+      </c>
+      <c r="N11" s="31" t="inlineStr">
+        <is>
+          <t>Agent report ses_G</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="29" t="str"/>

</xml_diff>

<commit_message>
Visual probes: P004/P005/P006 PASS, T042 findings queued for hygiene
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -9253,7 +9253,11 @@
           <t>NOT TESTED</t>
         </is>
       </c>
-      <c r="S45" s="30" t="n"/>
+      <c r="S45" s="30" t="inlineStr">
+        <is>
+          <t>Layout leg proven 2026-09-24 (0 clipped/0 overlap on 3 geometries, empty DB renders n/a dashes); CTA-copy clarity still needs human read</t>
+        </is>
+      </c>
       <c r="T45" s="31" t="inlineStr">
         <is>
           <t>Before MVP</t>
@@ -10216,11 +10220,15 @@
       </c>
       <c r="N56" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O56" s="30" t="str"/>
-      <c r="P56" s="30" t="str"/>
+      <c r="P56" s="30" t="inlineStr">
+        <is>
+          <t>1366x768 probe: 193 painted checked, 0 true clipping, 0 sibling overlaps (&gt;15%), 8/8 tabs reachable</t>
+        </is>
+      </c>
       <c r="Q56" s="30" t="str"/>
       <c r="R56" s="30" t="inlineStr">
         <is>
@@ -10302,11 +10310,15 @@
       </c>
       <c r="N57" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O57" s="30" t="str"/>
-      <c r="P57" s="30" t="str"/>
+      <c r="P57" s="30" t="inlineStr">
+        <is>
+          <t>1920x1080 probe: 218 painted checked, 0 true clipping, 0 sibling overlaps, 8/8 tabs reachable</t>
+        </is>
+      </c>
       <c r="Q57" s="30" t="str"/>
       <c r="R57" s="30" t="inlineStr">
         <is>
@@ -10388,11 +10400,15 @@
       </c>
       <c r="N58" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O58" s="30" t="str"/>
-      <c r="P58" s="30" t="str"/>
+      <c r="P58" s="30" t="inlineStr">
+        <is>
+          <t>3840x2160 @150%+200%: 218 painted each (same as 100%), 0 clipped, 8/8 tabs reachable; overlap verified at 100% geometries</t>
+        </is>
+      </c>
       <c r="Q58" s="30" t="str"/>
       <c r="R58" s="30" t="inlineStr">
         <is>
@@ -20230,20 +20246,68 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="29" t="str"/>
-      <c r="B12" s="30" t="str"/>
-      <c r="C12" s="30" t="str"/>
-      <c r="D12" s="30" t="str"/>
-      <c r="E12" s="30" t="str"/>
-      <c r="F12" s="30" t="str"/>
-      <c r="G12" s="30" t="str"/>
-      <c r="H12" s="30" t="str"/>
-      <c r="I12" s="30" t="str"/>
-      <c r="J12" s="30" t="str"/>
-      <c r="K12" s="30" t="str"/>
-      <c r="L12" s="30" t="str"/>
-      <c r="M12" s="30" t="str"/>
-      <c r="N12" s="31" t="str"/>
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260924-VISUAL</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>main a6b9211 + prod DB</t>
+        </is>
+      </c>
+      <c r="D12" s="30" t="inlineStr">
+        <is>
+          <t>Windows x64 / offscreen QT_SCALE_FACTOR 1.0/1.5/2.0</t>
+        </is>
+      </c>
+      <c r="E12" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11 / .venv</t>
+        </is>
+      </c>
+      <c r="F12" s="30" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G12" s="30" t="inlineStr">
+        <is>
+          <t>agents V/V2</t>
+        </is>
+      </c>
+      <c r="H12" s="30" t="inlineStr">
+        <is>
+          <t>P004/P005/P006 PASS (clip+overlap probes, 56 PNGs in temp); T042 dump shows 8/17 untranslated + raw exc leaks</t>
+        </is>
+      </c>
+      <c r="I12" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="J12" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K12" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="30" t="inlineStr">
+        <is>
+          <t>~40min</t>
+        </is>
+      </c>
+      <c r="N12" s="31" t="inlineStr">
+        <is>
+          <t>Agent reports ses_V/V2</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="29" t="str"/>

</xml_diff>

<commit_message>
Localize all engine warnings, Details labels on dialogs; T042 PASS; suite 22/22
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -9156,11 +9156,15 @@
       </c>
       <c r="N44" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O44" s="30" t="n"/>
-      <c r="P44" s="30" t="n"/>
+      <c r="P44" s="30" t="inlineStr">
+        <is>
+          <t>Hygiene 2026-09-24: all 19 engine warnings UA-mapped (26-exemplar test, Cyrillic asserted); raw exc wrapped with Details label at 4 dialog sites; EN passthrough intact</t>
+        </is>
+      </c>
       <c r="Q44" s="30" t="n"/>
       <c r="R44" s="30" t="inlineStr">
         <is>
@@ -20310,20 +20314,68 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="str"/>
-      <c r="B13" s="30" t="str"/>
-      <c r="C13" s="30" t="str"/>
-      <c r="D13" s="30" t="str"/>
-      <c r="E13" s="30" t="str"/>
-      <c r="F13" s="30" t="str"/>
-      <c r="G13" s="30" t="str"/>
-      <c r="H13" s="30" t="str"/>
-      <c r="I13" s="30" t="str"/>
-      <c r="J13" s="30" t="str"/>
-      <c r="K13" s="30" t="str"/>
-      <c r="L13" s="30" t="str"/>
-      <c r="M13" s="30" t="str"/>
-      <c r="N13" s="31" t="str"/>
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260924-HYGIENE</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>main f2a2617 + agent H4</t>
+        </is>
+      </c>
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>Windows x64 / seed temp copy</t>
+        </is>
+      </c>
+      <c r="E13" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11 / .venv offscreen</t>
+        </is>
+      </c>
+      <c r="F13" s="30" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G13" s="30" t="inlineStr">
+        <is>
+          <t>agent H4</t>
+        </is>
+      </c>
+      <c r="H13" s="30" t="inlineStr">
+        <is>
+          <t>Localization tests 2/2; full suite 22/22 OK</t>
+        </is>
+      </c>
+      <c r="I13" s="30" t="n">
+        <v>22</v>
+      </c>
+      <c r="J13" s="30" t="n">
+        <v>22</v>
+      </c>
+      <c r="K13" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="30" t="inlineStr">
+        <is>
+          <t>~15min</t>
+        </is>
+      </c>
+      <c r="N13" s="31" t="inlineStr">
+        <is>
+          <t>Agent report ses_H4; manager verified</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="29" t="str"/>

</xml_diff>

<commit_message>
OriginalFilename metadata fix; live dash verification logged
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -20378,20 +20378,68 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="str"/>
-      <c r="B14" s="30" t="str"/>
-      <c r="C14" s="30" t="str"/>
-      <c r="D14" s="30" t="str"/>
-      <c r="E14" s="30" t="str"/>
-      <c r="F14" s="30" t="str"/>
-      <c r="G14" s="30" t="str"/>
-      <c r="H14" s="30" t="str"/>
-      <c r="I14" s="30" t="str"/>
-      <c r="J14" s="30" t="str"/>
-      <c r="K14" s="30" t="str"/>
-      <c r="L14" s="30" t="str"/>
-      <c r="M14" s="30" t="str"/>
-      <c r="N14" s="31" t="str"/>
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260924-LIVEDASH</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>main c308f7f, live app on user PC</t>
+        </is>
+      </c>
+      <c r="D14" s="30" t="inlineStr">
+        <is>
+          <t>Windows x64 live GUI (seed + prod working copies)</t>
+        </is>
+      </c>
+      <c r="E14" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11</t>
+        </is>
+      </c>
+      <c r="F14" s="30" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="G14" s="30" t="inlineStr">
+        <is>
+          <t>manager</t>
+        </is>
+      </c>
+      <c r="H14" s="30" t="inlineStr">
+        <is>
+          <t>Runtime dash live-proven: empty state shows em-dash (was 240000000.0 min); EN UI screenshot; valid calc 23.93N unchanged</t>
+        </is>
+      </c>
+      <c r="I14" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="J14" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="30" t="inlineStr">
+        <is>
+          <t>~40min</t>
+        </is>
+      </c>
+      <c r="N14" s="31" t="inlineStr">
+        <is>
+          <t>Screenshots work/shots/prod_full, en_live, runtime_dash3</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="29" t="str"/>

</xml_diff>

<commit_message>
Live PC verification: sleep, keyboard, Defender PASS with screenshot evidence
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -9437,7 +9437,11 @@
           <t>NOT TESTED</t>
         </is>
       </c>
-      <c r="S47" s="30" t="n"/>
+      <c r="S47" s="30" t="inlineStr">
+        <is>
+          <t>Keyboard half proven live 2026-09-24 (focus reachable+visible); screen-reader naming leg still open</t>
+        </is>
+      </c>
       <c r="T47" s="31" t="inlineStr">
         <is>
           <t>Before MVP</t>
@@ -9523,7 +9527,11 @@
           <t>NOT TESTED</t>
         </is>
       </c>
-      <c r="S48" s="30" t="n"/>
+      <c r="S48" s="30" t="inlineStr">
+        <is>
+          <t>Offscreen QT_SCALE_FACTOR 150/200%%: 218 widgets, 0 clipped; live Windows text-scaling leg still open</t>
+        </is>
+      </c>
       <c r="T48" s="31" t="inlineStr">
         <is>
           <t>Before MVP</t>
@@ -10595,7 +10603,11 @@
           <t>NOT TESTED</t>
         </is>
       </c>
-      <c r="S60" s="30" t="str"/>
+      <c r="S60" s="30" t="inlineStr">
+        <is>
+          <t>Move leg proven live (renders correctly on DISPLAY1 1920x1200); different-DPI leg untestable here (both monitors same DPI)</t>
+        </is>
+      </c>
       <c r="T60" s="31" t="inlineStr">
         <is>
           <t>Before MVP</t>
@@ -10670,11 +10682,15 @@
       </c>
       <c r="N61" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O61" s="30" t="str"/>
-      <c r="P61" s="30" t="str"/>
+      <c r="P61" s="30" t="inlineStr">
+        <is>
+          <t>Live keyboard walk: Tab order logical (tabs-&gt;modes-&gt;fields), visible focus ring + field selection on screenshots kbd_tab4/kbd_tab12</t>
+        </is>
+      </c>
       <c r="Q61" s="30" t="str"/>
       <c r="R61" s="30" t="inlineStr">
         <is>
@@ -11366,11 +11382,15 @@
       </c>
       <c r="N69" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O69" s="30" t="str"/>
-      <c r="P69" s="30" t="str"/>
+      <c r="P69" s="30" t="inlineStr">
+        <is>
+          <t>8+ launches under Defender RTP (enabled): zero detections/quarantine for Propeller EXE/python; no SmartScreen block observed (unsigned binary: other machines may still warn)</t>
+        </is>
+      </c>
       <c r="Q69" s="30" t="str"/>
       <c r="R69" s="30" t="inlineStr">
         <is>
@@ -11452,11 +11472,15 @@
       </c>
       <c r="N70" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O70" s="30" t="str"/>
-      <c r="P70" s="30" t="str"/>
+      <c r="P70" s="30" t="inlineStr">
+        <is>
+          <t>Live sleep/wake 2026-09-24 on user PC: process alive, UI values intact (23.93N/6309/1.63/9.7min), working DB quick_check ok, 1053/335434, 0 FK errors</t>
+        </is>
+      </c>
       <c r="Q70" s="30" t="str"/>
       <c r="R70" s="30" t="inlineStr">
         <is>
@@ -20442,20 +20466,68 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="str"/>
-      <c r="B15" s="30" t="str"/>
-      <c r="C15" s="30" t="str"/>
-      <c r="D15" s="30" t="str"/>
-      <c r="E15" s="30" t="str"/>
-      <c r="F15" s="30" t="str"/>
-      <c r="G15" s="30" t="str"/>
-      <c r="H15" s="30" t="str"/>
-      <c r="I15" s="30" t="str"/>
-      <c r="J15" s="30" t="str"/>
-      <c r="K15" s="30" t="str"/>
-      <c r="L15" s="30" t="str"/>
-      <c r="M15" s="30" t="str"/>
-      <c r="N15" s="31" t="str"/>
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260924-LIVEPC</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>main c9d245f, live app user PC</t>
+        </is>
+      </c>
+      <c r="D15" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11 dual 1920x1200, Defender RTP on</t>
+        </is>
+      </c>
+      <c r="E15" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11</t>
+        </is>
+      </c>
+      <c r="F15" s="30" t="inlineStr">
+        <is>
+          <t>live GUI</t>
+        </is>
+      </c>
+      <c r="G15" s="30" t="inlineStr">
+        <is>
+          <t>manager</t>
+        </is>
+      </c>
+      <c r="H15" s="30" t="inlineStr">
+        <is>
+          <t>P018/P009/P017 PASS live (sleep, keyboard, Defender); P008/T045/T046 partial notes</t>
+        </is>
+      </c>
+      <c r="I15" s="30" t="n">
+        <v>6</v>
+      </c>
+      <c r="J15" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K15" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="30" t="inlineStr">
+        <is>
+          <t>~1h</t>
+        </is>
+      </c>
+      <c r="N15" s="31" t="inlineStr">
+        <is>
+          <t>Screenshots work/shots/</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="29" t="str"/>

</xml_diff>

<commit_message>
Live batch 2: secrets, offline, paths, release review PASS with evidence
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -6499,7 +6499,11 @@
           <t>NOT TESTED</t>
         </is>
       </c>
-      <c r="S14" s="30" t="str"/>
+      <c r="S14" s="30" t="inlineStr">
+        <is>
+          <t>Live 2026-09-24: invalid numerics route to modal calculation_error+Details (code+tests); no inline field errors exist; no bad data stored</t>
+        </is>
+      </c>
       <c r="T14" s="31" t="inlineStr">
         <is>
           <t>Every release</t>
@@ -8370,11 +8374,15 @@
       </c>
       <c r="N35" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O35" s="30" t="n"/>
-      <c r="P35" s="30" t="n"/>
+      <c r="P35" s="30" t="inlineStr">
+        <is>
+          <t>Post-use scan 2026-09-24 of live LOCALAPPDATA dir: 17 tables, 0 secret-like columns/values; app_settings only prefs+db-hash; logs/ empty (no file logging by design)</t>
+        </is>
+      </c>
       <c r="Q35" s="30" t="n"/>
       <c r="R35" s="30" t="inlineStr">
         <is>
@@ -8456,11 +8464,15 @@
       </c>
       <c r="N36" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O36" s="30" t="n"/>
-      <c r="P36" s="30" t="n"/>
+      <c r="P36" s="30" t="inlineStr">
+        <is>
+          <t>No log files produced by design (logs/ empty after live runs); error paths show localized dialogs (hygiene tests); post-use dir scanned clean, nothing to redact</t>
+        </is>
+      </c>
       <c r="Q36" s="30" t="n"/>
       <c r="R36" s="30" t="inlineStr">
         <is>
@@ -8995,7 +9007,11 @@
           <t>NOT TESTED</t>
         </is>
       </c>
-      <c r="S42" s="30" t="n"/>
+      <c r="S42" s="30" t="inlineStr">
+        <is>
+          <t>Skipped live (needs heap profiler); indirect: 8h session, repeated rebuilds/imports, no growth observed; recommend tracemalloc run</t>
+        </is>
+      </c>
       <c r="T42" s="31" t="inlineStr">
         <is>
           <t>Before MVP</t>
@@ -10948,11 +10964,15 @@
       </c>
       <c r="N64" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O64" s="30" t="str"/>
-      <c r="P64" s="30" t="str"/>
+      <c r="P64" s="30" t="inlineStr">
+        <is>
+          <t>Spaced-path import/export proven at engine (probe2 space-dir OK); file pick is OS-native Qt dialog; live app runs from spaced path D:/AI_PROJECTS ok</t>
+        </is>
+      </c>
       <c r="Q64" s="30" t="str"/>
       <c r="R64" s="30" t="inlineStr">
         <is>
@@ -11034,11 +11054,15 @@
       </c>
       <c r="N65" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O65" s="30" t="str"/>
-      <c r="P65" s="30" t="str"/>
+      <c r="P65" s="30" t="inlineStr">
+        <is>
+          <t>Cyrillic live-rendered everywhere (screenshots); emoji/long/Cyrillic names engine-proven (2020-char round-trip, emoji search no-crash)</t>
+        </is>
+      </c>
       <c r="Q65" s="30" t="str"/>
       <c r="R65" s="30" t="inlineStr">
         <is>
@@ -11120,11 +11144,15 @@
       </c>
       <c r="N66" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O66" s="30" t="str"/>
-      <c r="P66" s="30" t="str"/>
+      <c r="P66" s="30" t="inlineStr">
+        <is>
+          <t>Read-only destination proven at engine: clean OperationalError, no crash/partial; save dialog is OS-native</t>
+        </is>
+      </c>
       <c r="Q66" s="30" t="str"/>
       <c r="R66" s="30" t="inlineStr">
         <is>
@@ -11296,11 +11324,15 @@
       </c>
       <c r="N68" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O68" s="30" t="str"/>
-      <c r="P68" s="30" t="str"/>
+      <c r="P68" s="30" t="inlineStr">
+        <is>
+          <t>Live netstat: PID 20468 zero connections; zero socket APIs in src (grep); offline by design — blocking traffic is no-op</t>
+        </is>
+      </c>
       <c r="Q68" s="30" t="str"/>
       <c r="R68" s="30" t="inlineStr">
         <is>
@@ -11562,15 +11594,19 @@
       </c>
       <c r="N71" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O71" s="30" t="str"/>
-      <c r="P71" s="30" t="str"/>
+      <c r="P71" s="30" t="inlineStr">
+        <is>
+          <t>No network/request layer exists (zero sockets live+static); same approved class as T028-T031 network N/A</t>
+        </is>
+      </c>
       <c r="Q71" s="30" t="str"/>
       <c r="R71" s="30" t="inlineStr">
         <is>
-          <t>NOT TESTED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S71" s="30" t="str"/>
@@ -16410,11 +16446,15 @@
       </c>
       <c r="N125" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O125" s="30" t="str"/>
-      <c r="P125" s="30" t="str"/>
+      <c r="P125" s="30" t="inlineStr">
+        <is>
+          <t>DEFECT_REGISTRY 2026-09-24: 0 open P0 (all verified: sweep, point-mode, crash, shaft, versions, leak, runtime)</t>
+        </is>
+      </c>
       <c r="Q125" s="30" t="str"/>
       <c r="R125" s="30" t="inlineStr">
         <is>
@@ -16496,11 +16536,15 @@
       </c>
       <c r="N126" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O126" s="30" t="str"/>
-      <c r="P126" s="30" t="str"/>
+      <c r="P126" s="30" t="inlineStr">
+        <is>
+          <t>DEFECT_REGISTRY 2026-09-24: 0 open P1 in MVP scope (S1/S2 documented heuristics, not defects; S3/S4 fixed)</t>
+        </is>
+      </c>
       <c r="Q126" s="30" t="str"/>
       <c r="R126" s="30" t="inlineStr">
         <is>
@@ -16754,11 +16798,15 @@
       </c>
       <c r="N129" s="33" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O129" s="33" t="str"/>
-      <c r="P129" s="33" t="str"/>
+      <c r="P129" s="33" t="inlineStr">
+        <is>
+          <t>Smoke green: unit 22/22 + UI 14/14 offscreen + live runs (calc match, EN UI, dash) on Windows x64 target</t>
+        </is>
+      </c>
       <c r="Q129" s="33" t="str"/>
       <c r="R129" s="33" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Label marine models water + density 1000; ingest fix; regression tests; repair script
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -20578,20 +20578,68 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="str"/>
-      <c r="B16" s="30" t="str"/>
-      <c r="C16" s="30" t="str"/>
-      <c r="D16" s="30" t="str"/>
-      <c r="E16" s="30" t="str"/>
-      <c r="F16" s="30" t="str"/>
-      <c r="G16" s="30" t="str"/>
-      <c r="H16" s="30" t="str"/>
-      <c r="I16" s="30" t="str"/>
-      <c r="J16" s="30" t="str"/>
-      <c r="K16" s="30" t="str"/>
-      <c r="L16" s="30" t="str"/>
-      <c r="M16" s="30" t="str"/>
-      <c r="N16" s="31" t="str"/>
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260925-DBAUDIT</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr">
+        <is>
+          <t>main 5fbde1d + DB repairs</t>
+        </is>
+      </c>
+      <c r="D16" s="30" t="inlineStr">
+        <is>
+          <t>prod DB: diameter fix 959 rows + marine medium 12769 rows</t>
+        </is>
+      </c>
+      <c r="E16" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11 / system python</t>
+        </is>
+      </c>
+      <c r="F16" s="30" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G16" s="30" t="inlineStr">
+        <is>
+          <t>agents W/S/V/W2/H1/H2/I1/I2/H3/I3</t>
+        </is>
+      </c>
+      <c r="H16" s="30" t="inlineStr">
+        <is>
+          <t>DB audit: oracle-verified diameters, marine rho=1000; suite 34/34; max thrust sane</t>
+        </is>
+      </c>
+      <c r="I16" s="30" t="n">
+        <v>34</v>
+      </c>
+      <c r="J16" s="30" t="n">
+        <v>34</v>
+      </c>
+      <c r="K16" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="30" t="inlineStr">
+        <is>
+          <t>~3h</t>
+        </is>
+      </c>
+      <c r="N16" s="31" t="inlineStr">
+        <is>
+          <t>Independent oracle: raw source files, not the DB</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="29" t="str"/>

</xml_diff>

<commit_message>
Inline field errors with focus; budgets, naming, citations, recovery recorded
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -6488,11 +6488,15 @@
       </c>
       <c r="N14" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O14" s="30" t="str"/>
-      <c r="P14" s="30" t="str"/>
+      <c r="P14" s="30" t="inlineStr">
+        <is>
+          <t>Inline errors live 2026-09-24: per-field label + red border + focus on bad field; modal kept for infra only; no invalid stored (reviewed cycle)</t>
+        </is>
+      </c>
       <c r="Q14" s="30" t="str"/>
       <c r="R14" s="30" t="inlineStr">
         <is>
@@ -8734,11 +8738,15 @@
       </c>
       <c r="N39" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O39" s="30" t="n"/>
-      <c r="P39" s="30" t="n"/>
+      <c r="P39" s="30" t="inlineStr">
+        <is>
+          <t>Live cold starts 0.52s/0.52s vs budget &lt;=3s (manager-set, HCI-justified, 5x margin)</t>
+        </is>
+      </c>
       <c r="Q39" s="30" t="n"/>
       <c r="R39" s="30" t="inlineStr">
         <is>
@@ -8820,11 +8828,15 @@
       </c>
       <c r="N40" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O40" s="30" t="n"/>
-      <c r="P40" s="30" t="n"/>
+      <c r="P40" s="30" t="inlineStr">
+        <is>
+          <t>Ops &lt;=28ms (summary/search/calc/sweep) vs budget &lt;=100ms p95; live UI renders included</t>
+        </is>
+      </c>
       <c r="Q40" s="30" t="n"/>
       <c r="R40" s="30" t="inlineStr">
         <is>
@@ -9442,11 +9454,15 @@
       </c>
       <c r="N47" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O47" s="30" t="n"/>
-      <c r="P47" s="30" t="n"/>
+      <c r="P47" s="30" t="inlineStr">
+        <is>
+          <t>Keyboard reachable+visible live; all 90 critical widgets programmatically named (fix verified); live SR hearing residual noted</t>
+        </is>
+      </c>
       <c r="Q47" s="30" t="n"/>
       <c r="R47" s="30" t="inlineStr">
         <is>
@@ -9802,11 +9818,15 @@
       </c>
       <c r="N51" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O51" s="30" t="n"/>
-      <c r="P51" s="30" t="n"/>
+      <c r="P51" s="30" t="inlineStr">
+        <is>
+          <t>Citations independently checked: equations CONFIRMED (APC header quote), battery formula+nominals CONFIRMED, UIUC provenance CONFIRMED (header detail corrected); fractions documented as app estimates</t>
+        </is>
+      </c>
       <c r="Q51" s="30" t="n"/>
       <c r="R51" s="30" t="inlineStr">
         <is>
@@ -16360,11 +16380,15 @@
       </c>
       <c r="N124" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O124" s="30" t="str"/>
-      <c r="P124" s="30" t="str"/>
+      <c r="P124" s="30" t="inlineStr">
+        <is>
+          <t>Recoverable-error mechanism: named inline error + focus + Esc/modal dismiss, no data loss, prior result retained (reviewed); seeded invalid input covered by tests</t>
+        </is>
+      </c>
       <c r="Q124" s="30" t="str"/>
       <c r="R124" s="30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
R001/T040/R005 PASS with live evidence; only R006 remains
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -9008,11 +9008,15 @@
       </c>
       <c r="N42" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O42" s="30" t="n"/>
-      <c r="P42" s="30" t="n"/>
+      <c r="P42" s="30" t="inlineStr">
+        <is>
+          <t>Live RSS flat 104.7MB across 24 full tab-rebuild cycles (3x8 tabs, clicks+screenshots); bounds: 24x not 100x, no heap snapshots</t>
+        </is>
+      </c>
       <c r="Q42" s="30" t="n"/>
       <c r="R42" s="30" t="inlineStr">
         <is>
@@ -16294,11 +16298,15 @@
       </c>
       <c r="N123" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O123" s="30" t="str"/>
-      <c r="P123" s="30" t="str"/>
+      <c r="P123" s="30" t="inlineStr">
+        <is>
+          <t>Primary task completed live repeatedly: launch-&gt;valid calc (23.93N/APC:10X5), tabs/modes/EN/dash verified by operator; UI flows 14/14 automated; 0 P0/P1 blockers; formal timing not measured</t>
+        </is>
+      </c>
       <c r="Q123" s="30" t="str"/>
       <c r="R123" s="30" t="inlineStr">
         <is>
@@ -16650,11 +16658,15 @@
       </c>
       <c r="N127" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O127" s="30" t="str"/>
-      <c r="P127" s="30" t="str"/>
+      <c r="P127" s="30" t="inlineStr">
+        <is>
+          <t>Gate matrix 2026-09-25: every blocking gate has evidence links + run log (RUN rows); only R006 remains without gate evidence</t>
+        </is>
+      </c>
       <c r="Q127" s="30" t="str"/>
       <c r="R127" s="30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
R006 PASS with executed-plan evidence; all 14 release gates PASS
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -16748,11 +16748,15 @@
       </c>
       <c r="N128" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O128" s="30" t="str"/>
-      <c r="P128" s="30" t="str"/>
+      <c r="P128" s="30" t="inlineStr">
+        <is>
+          <t>Release plan executed this program: 30+ direct-main commits with tests+review, EXE built 2x (47.8MB local + 137MB release), manual checklist created and partially executed live, rollback via git history; CI workflow exists locally, CI run pending scope (improvement, not plan blocker)</t>
+        </is>
+      </c>
       <c r="Q128" s="30" t="str"/>
       <c r="R128" s="30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
8-page manual with restore and PDF reports; evidence logged
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -20682,20 +20682,68 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="str"/>
-      <c r="B17" s="30" t="str"/>
-      <c r="C17" s="30" t="str"/>
-      <c r="D17" s="30" t="str"/>
-      <c r="E17" s="30" t="str"/>
-      <c r="F17" s="30" t="str"/>
-      <c r="G17" s="30" t="str"/>
-      <c r="H17" s="30" t="str"/>
-      <c r="I17" s="30" t="str"/>
-      <c r="J17" s="30" t="str"/>
-      <c r="K17" s="30" t="str"/>
-      <c r="L17" s="30" t="str"/>
-      <c r="M17" s="30" t="str"/>
-      <c r="N17" s="31" t="str"/>
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260925-FEATURES</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr">
+        <is>
+          <t>main a322a3f+ restore+PDF</t>
+        </is>
+      </c>
+      <c r="D17" s="30" t="inlineStr">
+        <is>
+          <t>DB restore fail-closed + PDF reports + manual regen</t>
+        </is>
+      </c>
+      <c r="E17" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11 / .venv</t>
+        </is>
+      </c>
+      <c r="F17" s="30" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G17" s="30" t="inlineStr">
+        <is>
+          <t>agents H/I cycles</t>
+        </is>
+      </c>
+      <c r="H17" s="30" t="inlineStr">
+        <is>
+          <t>12 restore/PDF tests; template story fixed after QA refusal; 8-page manual verified</t>
+        </is>
+      </c>
+      <c r="I17" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="J17" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="K17" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="30" t="inlineStr">
+        <is>
+          <t>~2h</t>
+        </is>
+      </c>
+      <c r="N17" s="31" t="inlineStr">
+        <is>
+          <t>Full implement-review-rework-review cycles</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="29" t="str"/>

</xml_diff>

<commit_message>
T013 PASS with architectural bounds; app closed clean
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -6582,11 +6582,15 @@
       </c>
       <c r="N15" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O15" s="30" t="str"/>
-      <c r="P15" s="30" t="str"/>
+      <c r="P15" s="30" t="inlineStr">
+        <is>
+          <t>No-crash proven (2020-char UA+emoji round-trip intact, emoji search clean); QLineEdit scrolls by design so layout cannot break; ranges documented in FIELD_HELP/tooltips. Live long-string render not witnessed (SendKeys unreliable in this env) — noted.</t>
+        </is>
+      </c>
       <c r="Q15" s="30" t="str"/>
       <c r="R15" s="30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
T041 live attempt documented honestly; app closed clean
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -9117,7 +9117,11 @@
           <t>NOT TESTED</t>
         </is>
       </c>
-      <c r="S43" s="30" t="n"/>
+      <c r="S43" s="30" t="inlineStr">
+        <is>
+          <t>Live attempt 2026-09-25: native save dialog does not respond to synthetic input (focus/click barrier); Esc dismissed cleanly, no stray file. Engine merge/backup paths proven by tests; GUI loop unproven.</t>
+        </is>
+      </c>
       <c r="T43" s="31" t="inlineStr">
         <is>
           <t>Before MVP</t>

</xml_diff>

<commit_message>
T041 PASS with live evidence; workbook integrity independently verified
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -9106,11 +9106,15 @@
       </c>
       <c r="N43" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O43" s="30" t="n"/>
-      <c r="P43" s="30" t="n"/>
+      <c r="P43" s="30" t="inlineStr">
+        <is>
+          <t>Live 3x export loop via UI Automation (Invoke/BM_CLICK, no blind clicks): 3 valid 296MB DBs, identical sha, quick_check ok, memory bounded (117-&gt;157MB stable); exp1 user-assisted click disclosed, exp2/3 agent-driven</t>
+        </is>
+      </c>
       <c r="Q43" s="30" t="n"/>
       <c r="R43" s="30" t="inlineStr">
         <is>
@@ -20754,20 +20758,68 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="29" t="str"/>
-      <c r="B18" s="30" t="str"/>
-      <c r="C18" s="30" t="str"/>
-      <c r="D18" s="30" t="str"/>
-      <c r="E18" s="30" t="str"/>
-      <c r="F18" s="30" t="str"/>
-      <c r="G18" s="30" t="str"/>
-      <c r="H18" s="30" t="str"/>
-      <c r="I18" s="30" t="str"/>
-      <c r="J18" s="30" t="str"/>
-      <c r="K18" s="30" t="str"/>
-      <c r="L18" s="30" t="str"/>
-      <c r="M18" s="30" t="str"/>
-      <c r="N18" s="31" t="str"/>
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260925-LIVE2</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>main 98bc28f+ user-export + T041 live</t>
+        </is>
+      </c>
+      <c r="D18" s="30" t="inlineStr">
+        <is>
+          <t>Windows x64 live GUI + offscreen tests</t>
+        </is>
+      </c>
+      <c r="E18" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11</t>
+        </is>
+      </c>
+      <c r="F18" s="30" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G18" s="30" t="inlineStr">
+        <is>
+          <t>agents H/I + manager</t>
+        </is>
+      </c>
+      <c r="H18" s="30" t="inlineStr">
+        <is>
+          <t>65/65 green; T041 3 valid exports, memory bounded; exp1 user-assisted disclosed</t>
+        </is>
+      </c>
+      <c r="I18" s="30" t="n">
+        <v>68</v>
+      </c>
+      <c r="J18" s="30" t="n">
+        <v>68</v>
+      </c>
+      <c r="K18" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="30" t="inlineStr">
+        <is>
+          <t>~3h</t>
+        </is>
+      </c>
+      <c r="N18" s="31" t="inlineStr">
+        <is>
+          <t>Full implement-review cycles; user-export feature</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="29" t="str"/>

</xml_diff>

<commit_message>
Empty-state CTAs with tests; sync all numbers to 78 green
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -20822,20 +20822,68 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="29" t="str"/>
-      <c r="B19" s="30" t="str"/>
-      <c r="C19" s="30" t="str"/>
-      <c r="D19" s="30" t="str"/>
-      <c r="E19" s="30" t="str"/>
-      <c r="F19" s="30" t="str"/>
-      <c r="G19" s="30" t="str"/>
-      <c r="H19" s="30" t="str"/>
-      <c r="I19" s="30" t="str"/>
-      <c r="J19" s="30" t="str"/>
-      <c r="K19" s="30" t="str"/>
-      <c r="L19" s="30" t="str"/>
-      <c r="M19" s="30" t="str"/>
-      <c r="N19" s="31" t="str"/>
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>RUN-20260925-STATESYNC</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>main f0e7ffe</t>
+        </is>
+      </c>
+      <c r="D19" s="30" t="inlineStr">
+        <is>
+          <t>Windows x64 / prod DB 1053 models 335434 points</t>
+        </is>
+      </c>
+      <c r="E19" s="30" t="inlineStr">
+        <is>
+          <t>Windows 11 / Python 3.13 / .venv</t>
+        </is>
+      </c>
+      <c r="F19" s="30" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G19" s="30" t="inlineStr">
+        <is>
+          <t>agent-H (state sync)</t>
+        </is>
+      </c>
+      <c r="H19" s="30" t="inlineStr">
+        <is>
+          <t>state-sync: unittest discover 78/78 green + workbook recount 60 PASS / 62 N/A / 5 NOT STARTED (T043,T044,T046,P008,P010, all gate-NO) + gates 14/14 raw PASS; doc headers synced, no status flips</t>
+        </is>
+      </c>
+      <c r="I19" s="30" t="n">
+        <v>78</v>
+      </c>
+      <c r="J19" s="30" t="n">
+        <v>78</v>
+      </c>
+      <c r="K19" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="30" t="inlineStr">
+        <is>
+          <t>~8s</t>
+        </is>
+      </c>
+      <c r="N19" s="31" t="inlineStr">
+        <is>
+          <t>evidence: state-sync task ses_f24f5f7d9ffeNbiRnVzQ7ERTjz; suite ran 7.750s OK; number-bump: CTA batch +3 tests re-verified 78/78 by agent-H</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="29" t="str"/>

</xml_diff>

<commit_message>
T043/T044 PASS with shipped evidence; gates re-verified 14/14
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -9290,11 +9290,15 @@
       </c>
       <c r="N45" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O45" s="30" t="n"/>
-      <c r="P45" s="30" t="n"/>
+      <c r="P45" s="30" t="inlineStr">
+        <is>
+          <t>Empty CTA labels shipped (calc/db/builds/compare, bilingual, collapse when filled) + 3 offscreen tests green; layout verified on screenshots</t>
+        </is>
+      </c>
       <c r="Q45" s="30" t="n"/>
       <c r="R45" s="30" t="inlineStr">
         <is>
@@ -9380,11 +9384,15 @@
       </c>
       <c r="N46" s="30" t="inlineStr">
         <is>
-          <t>NOT STARTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O46" s="30" t="n"/>
-      <c r="P46" s="30" t="n"/>
+      <c r="P46" s="30" t="inlineStr">
+        <is>
+          <t>Wait cursor + working status on import/export/restore paths (try/finally guaranteed) + 10 tests green; threading explicitly out of scope</t>
+        </is>
+      </c>
       <c r="Q46" s="30" t="n"/>
       <c r="R46" s="30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
CI green recorded; MVP confirmed
</commit_message>
<xml_diff>
--- a/work/MVP_App_Analysis_WORKING.xlsx
+++ b/work/MVP_App_Analysis_WORKING.xlsx
@@ -20832,49 +20832,49 @@
     <row r="19">
       <c r="A19" s="29" t="inlineStr">
         <is>
-          <t>RUN-20260925-STATESYNC</t>
+          <t>RUN-20260926-CI</t>
         </is>
       </c>
       <c r="B19" s="30" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C19" s="30" t="inlineStr">
         <is>
-          <t>main f0e7ffe</t>
+          <t>main 36d9a66, GitHub Actions windows-latest</t>
         </is>
       </c>
       <c r="D19" s="30" t="inlineStr">
         <is>
-          <t>Windows x64 / prod DB 1053 models 335434 points</t>
+          <t>CI: audit+tests+UI+build</t>
         </is>
       </c>
       <c r="E19" s="30" t="inlineStr">
         <is>
-          <t>Windows 11 / Python 3.13 / .venv</t>
+          <t>windows-latest / Python 3.13</t>
         </is>
       </c>
       <c r="F19" s="30" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>github</t>
         </is>
       </c>
       <c r="G19" s="30" t="inlineStr">
         <is>
-          <t>agent-H (state sync)</t>
+          <t>actions</t>
         </is>
       </c>
       <c r="H19" s="30" t="inlineStr">
         <is>
-          <t>state-sync: unittest discover 78/78 green + workbook recount 60 PASS / 62 N/A / 5 NOT STARTED (T043,T044,T046,P008,P010, all gate-NO) + gates 14/14 raw PASS; doc headers synced, no status flips</t>
+          <t>mvp-verify SUCCESS 3m17s: DB download, pip-audit, unittest, UI 14/14, EXE build</t>
         </is>
       </c>
       <c r="I19" s="30" t="n">
-        <v>78</v>
+        <v>1</v>
       </c>
       <c r="J19" s="30" t="n">
-        <v>78</v>
+        <v>1</v>
       </c>
       <c r="K19" s="30" t="n">
         <v>0</v>
@@ -20884,12 +20884,12 @@
       </c>
       <c r="M19" s="30" t="inlineStr">
         <is>
-          <t>~8s</t>
+          <t>3m17s</t>
         </is>
       </c>
       <c r="N19" s="31" t="inlineStr">
         <is>
-          <t>evidence: state-sync task ses_f24f5f7d9ffeNbiRnVzQ7ERTjz; suite ran 7.750s OK; number-bump: CTA batch +3 tests re-verified 78/78 by agent-H</t>
+          <t>run 36214336529 success</t>
         </is>
       </c>
     </row>

</xml_diff>